<commit_message>
Separate files for Stamp and Sproat Coho
</commit_message>
<xml_diff>
--- a/End-of-season Historic escapement files/Daily Totals by Age 2026 Example.xlsx
+++ b/End-of-season Historic escapement files/Daily Totals by Age 2026 Example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\POURFARAJV\Documents\GitHub\Somass-escapement-plots\End-of-season Historic escapement files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2499C384-405D-4986-A483-061935F37E87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9404AA6B-19D1-46A7-99E2-087FA8B8F09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sproat" sheetId="1" r:id="rId1"/>
@@ -24675,30 +24675,14 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A136" s="10"/>
-      <c r="B136" s="14">
-        <v>312</v>
-      </c>
-      <c r="C136" s="14">
-        <v>24</v>
-      </c>
-      <c r="D136" s="14">
-        <v>0</v>
-      </c>
-      <c r="E136" s="14">
-        <v>0</v>
-      </c>
-      <c r="F136" s="14">
-        <v>256</v>
-      </c>
-      <c r="G136" s="14">
-        <v>14</v>
-      </c>
-      <c r="H136" s="14">
-        <v>714.5</v>
-      </c>
-      <c r="I136" s="14">
-        <v>16</v>
-      </c>
+      <c r="B136" s="14"/>
+      <c r="C136" s="14"/>
+      <c r="D136" s="14"/>
+      <c r="E136" s="14"/>
+      <c r="F136" s="14"/>
+      <c r="G136" s="14"/>
+      <c r="H136" s="14"/>
+      <c r="I136" s="14"/>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137" s="10"/>

</xml_diff>